<commit_message>
Ready for large-scale teste
</commit_message>
<xml_diff>
--- a/tools/comparison_outputs/Alta_Lisboa_radiation_comparison.xlsx
+++ b/tools/comparison_outputs/Alta_Lisboa_radiation_comparison.xlsx
@@ -195,7 +195,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>30364.06000000001</v>
+        <v>30344.070000000003</v>
       </c>
     </row>
     <row r="16">
@@ -225,7 +225,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>50947617.550000004</v>
+        <v>50621829.330000006</v>
       </c>
     </row>
     <row r="19">
@@ -235,7 +235,7 @@
         </is>
       </c>
       <c r="B19">
-        <v>50909874.920000024</v>
+        <v>50542339.160000026</v>
       </c>
     </row>
     <row r="20">
@@ -245,7 +245,7 @@
         </is>
       </c>
       <c r="B20">
-        <v>-26.728263196077652</v>
+        <v>-27.19680460895591</v>
       </c>
     </row>
     <row r="21">
@@ -255,7 +255,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>-26.782543811828376</v>
+        <v>-27.311125613446873</v>
       </c>
     </row>
   </sheetData>
@@ -419,7 +419,7 @@
         <v>316.63596337502787</v>
       </c>
       <c r="E2">
-        <v>319.51</v>
+        <v>320.23</v>
       </c>
       <c r="F2">
         <v>316.6</v>
@@ -428,16 +428,16 @@
         <v>722452.69621875</v>
       </c>
       <c r="H2">
-        <v>539961.5199999999</v>
+        <v>518469.0</v>
       </c>
       <c r="I2">
-        <v>514414.79999999935</v>
+        <v>506833.9000000004</v>
       </c>
       <c r="J2">
-        <v>-0.2879605783293516</v>
+        <v>-0.2984538605050244</v>
       </c>
       <c r="K2">
-        <v>-0.2525994811478895</v>
+        <v>-0.2823488614360243</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -485,7 +485,7 @@
         <v>0.6940101385116577</v>
       </c>
       <c r="X2">
-        <v>0.634689014100703</v>
+        <v>0.633941413094328</v>
       </c>
       <c r="Y2">
         <v>0.4489450454711914</v>
@@ -523,16 +523,16 @@
         <v>6461016.0353125</v>
       </c>
       <c r="H3">
-        <v>5279354.109999982</v>
+        <v>5279842.170000022</v>
       </c>
       <c r="I3">
-        <v>5279952.880000014</v>
+        <v>5278975.140000027</v>
       </c>
       <c r="J3">
-        <v>-0.1827983631146276</v>
+        <v>-0.1829496922546024</v>
       </c>
       <c r="K3">
-        <v>-0.1828910373932178</v>
+        <v>-0.18281549819050213</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
         <v>2151885.359375</v>
       </c>
       <c r="H4">
-        <v>1633554.3200000057</v>
+        <v>1636518.369999998</v>
       </c>
       <c r="I4">
-        <v>1633098.3799999994</v>
+        <v>1637562.1700000037</v>
       </c>
       <c r="J4">
-        <v>-0.24108485943028052</v>
+        <v>-0.23901049706680375</v>
       </c>
       <c r="K4">
-        <v>-0.24087298011337369</v>
+        <v>-0.2394955600816424</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
         <v>183.52575815737313</v>
       </c>
       <c r="E5">
-        <v>180.52</v>
+        <v>186.33</v>
       </c>
       <c r="F5">
         <v>185.7</v>
@@ -683,16 +683,16 @@
         <v>382455.332625</v>
       </c>
       <c r="H5">
-        <v>307023.2399999995</v>
+        <v>316170.53999999934</v>
       </c>
       <c r="I5">
-        <v>320436.45</v>
+        <v>320501.34999999945</v>
       </c>
       <c r="J5">
-        <v>-0.1621598062166645</v>
+        <v>-0.1619901131977334</v>
       </c>
       <c r="K5">
-        <v>-0.19723111744126764</v>
+        <v>-0.17331381463569062</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
         <v>0.6830049157142639</v>
       </c>
       <c r="X5">
-        <v>0.6836608447089686</v>
+        <v>0.6834668882560337</v>
       </c>
       <c r="Y5">
         <v>0.6775040626525879</v>
@@ -778,16 +778,16 @@
         <v>1041488.901328125</v>
       </c>
       <c r="H6">
-        <v>880636.9800000046</v>
+        <v>880874.4600000061</v>
       </c>
       <c r="I6">
-        <v>880725.7300000016</v>
+        <v>881577.9700000011</v>
       </c>
       <c r="J6">
-        <v>-0.1543589865654021</v>
+        <v>-0.15354069652033991</v>
       </c>
       <c r="K6">
-        <v>-0.15444420110766344</v>
+        <v>-0.15421618139502066</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -858,16 +858,16 @@
         <v>365252.92209375004</v>
       </c>
       <c r="H7">
-        <v>295944.91999999963</v>
+        <v>295641.5800000002</v>
       </c>
       <c r="I7">
-        <v>295766.63999999897</v>
+        <v>295903.55000000034</v>
       </c>
       <c r="J7">
-        <v>-0.19024155014402847</v>
+        <v>-0.1898667139915439</v>
       </c>
       <c r="K7">
-        <v>-0.18975345001062308</v>
+        <v>-0.19058394302423293</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -938,16 +938,16 @@
         <v>10438925.579078125</v>
       </c>
       <c r="H8">
-        <v>7525957.809999977</v>
+        <v>7527267.299999986</v>
       </c>
       <c r="I8">
-        <v>7524601.990000011</v>
+        <v>7528021.740000001</v>
       </c>
       <c r="J8">
-        <v>-0.2791785004118672</v>
+        <v>-0.2788509044371585</v>
       </c>
       <c r="K8">
-        <v>-0.2790486192292019</v>
+        <v>-0.2789231762427481</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -1018,16 +1018,16 @@
         <v>1014674.485625</v>
       </c>
       <c r="H9">
-        <v>689365.6999999996</v>
+        <v>583640.0799999958</v>
       </c>
       <c r="I9">
-        <v>688799.9100000015</v>
+        <v>581515.3199999998</v>
       </c>
       <c r="J9">
-        <v>-0.3211616929780908</v>
+        <v>-0.4268947054071148</v>
       </c>
       <c r="K9">
-        <v>-0.3206040855798427</v>
+        <v>-0.4248006742374169</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -1098,16 +1098,16 @@
         <v>3759624.0890078126</v>
       </c>
       <c r="H10">
-        <v>2789762.56999999</v>
+        <v>2790138.3700000043</v>
       </c>
       <c r="I10">
-        <v>2789624.430000003</v>
+        <v>2790202.2500000084</v>
       </c>
       <c r="J10">
-        <v>-0.2580044270499922</v>
+        <v>-0.2578507361526243</v>
       </c>
       <c r="K10">
-        <v>-0.2579676840148598</v>
+        <v>-0.25786772721303136</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -1178,16 +1178,16 @@
         <v>1449804.290203125</v>
       </c>
       <c r="H11">
-        <v>1287157.4100000015</v>
+        <v>1286705.5500000021</v>
       </c>
       <c r="I11">
-        <v>1287503.8899999992</v>
+        <v>1286280.1700000032</v>
       </c>
       <c r="J11">
-        <v>-0.11194642014777503</v>
+        <v>-0.1127904788998874</v>
       </c>
       <c r="K11">
-        <v>-0.11218540412812254</v>
+        <v>-0.11249707378109074</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         <v>378.38995699688985</v>
       </c>
       <c r="E12">
-        <v>378.38</v>
+        <v>378.39</v>
       </c>
       <c r="F12">
         <v>378.38</v>
@@ -1258,16 +1258,16 @@
         <v>951905.74384375</v>
       </c>
       <c r="H12">
-        <v>625601.8699999992</v>
+        <v>604449.2500000014</v>
       </c>
       <c r="I12">
-        <v>627903.4000000013</v>
+        <v>620533.6100000007</v>
       </c>
       <c r="J12">
-        <v>-0.34037229624799054</v>
+        <v>-0.3481144388368584</v>
       </c>
       <c r="K12">
-        <v>-0.3427901091615976</v>
+        <v>-0.3650114479199756</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         <v>0.9890090823173523</v>
       </c>
       <c r="X12">
-        <v>0.9890090823173523</v>
+        <v>0.9890090823173522</v>
       </c>
       <c r="Y12">
         <v>0.9890090823173523</v>
@@ -1353,16 +1353,16 @@
         <v>1432575.848921875</v>
       </c>
       <c r="H13">
-        <v>1078085.9100000006</v>
+        <v>1076775.0300000021</v>
       </c>
       <c r="I13">
-        <v>1078304.2700000012</v>
+        <v>1076818.63</v>
       </c>
       <c r="J13">
-        <v>-0.24729690870364093</v>
+        <v>-0.2483339497797692</v>
       </c>
       <c r="K13">
-        <v>-0.24744933344273234</v>
+        <v>-0.24836438446846687</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         <v>735.2452728248661</v>
       </c>
       <c r="E14">
-        <v>734.71</v>
+        <v>735.19</v>
       </c>
       <c r="F14">
         <v>732.46</v>
@@ -1433,16 +1433,16 @@
         <v>1445044.5366953125</v>
       </c>
       <c r="H14">
-        <v>1272632.4800000037</v>
+        <v>1269531.9600000018</v>
       </c>
       <c r="I14">
-        <v>1270517.9199999978</v>
+        <v>1271310.7799999965</v>
       </c>
       <c r="J14">
-        <v>-0.1207759430684686</v>
+        <v>-0.12022726793779623</v>
       </c>
       <c r="K14">
-        <v>-0.11931262484795085</v>
+        <v>-0.12145824729851733</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
         <v>0.9921562671661377</v>
       </c>
       <c r="X14">
-        <v>0.9921562671661377</v>
+        <v>0.9921562671661378</v>
       </c>
       <c r="Y14">
         <v>0.9921562671661377</v>
@@ -1528,16 +1528,16 @@
         <v>1096379.78125</v>
       </c>
       <c r="H15">
-        <v>743965.810000001</v>
+        <v>748999.5700000013</v>
       </c>
       <c r="I15">
-        <v>746862.0799999982</v>
+        <v>751955.3599999994</v>
       </c>
       <c r="J15">
-        <v>-0.3187925454549254</v>
+        <v>-0.31414700192420264</v>
       </c>
       <c r="K15">
-        <v>-0.32143421219260926</v>
+        <v>-0.3168429564196678</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
         <v>503.4881674734263</v>
       </c>
       <c r="E16">
-        <v>497.04</v>
+        <v>503.36</v>
       </c>
       <c r="F16">
         <v>491.6</v>
@@ -1608,16 +1608,16 @@
         <v>1165644.1205625</v>
       </c>
       <c r="H16">
-        <v>862701.0899999981</v>
+        <v>874399.0099999972</v>
       </c>
       <c r="I16">
-        <v>853288.3800000006</v>
+        <v>853052.6100000005</v>
       </c>
       <c r="J16">
-        <v>-0.26796835762511056</v>
+        <v>-0.2681706234761032</v>
       </c>
       <c r="K16">
-        <v>-0.2598932429018833</v>
+        <v>-0.24985765846093566</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
         <v>1269227.792875</v>
       </c>
       <c r="H17">
-        <v>971308.1000000042</v>
+        <v>971190.2700000006</v>
       </c>
       <c r="I17">
-        <v>970665.6400000021</v>
+        <v>971713.6699999991</v>
       </c>
       <c r="J17">
-        <v>-0.2352313387329061</v>
+        <v>-0.23440561619052225</v>
       </c>
       <c r="K17">
-        <v>-0.23472515693984375</v>
+        <v>-0.23481799291512337</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1783,16 +1783,16 @@
         <v>934826.555390625</v>
       </c>
       <c r="H18">
-        <v>671672.1199999972</v>
+        <v>670144.4500000004</v>
       </c>
       <c r="I18">
-        <v>671548.7300000011</v>
+        <v>669498.8300000005</v>
       </c>
       <c r="J18">
-        <v>-0.2816328054358822</v>
+        <v>-0.2838256186247887</v>
       </c>
       <c r="K18">
-        <v>-0.2815008130365601</v>
+        <v>-0.28313498783742297</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1863,16 +1863,16 @@
         <v>516489.6829375</v>
       </c>
       <c r="H19">
-        <v>366093.43</v>
+        <v>397324.46000000014</v>
       </c>
       <c r="I19">
-        <v>365949.16999999905</v>
+        <v>397802.26999999984</v>
       </c>
       <c r="J19">
-        <v>-0.291468577031998</v>
+        <v>-0.22979628995195714</v>
       </c>
       <c r="K19">
-        <v>-0.2911892684518528</v>
+        <v>-0.23072140039614297</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1943,16 +1943,16 @@
         <v>1100404.8786875</v>
       </c>
       <c r="H20">
-        <v>784224.1900000022</v>
+        <v>772873.0300000012</v>
       </c>
       <c r="I20">
-        <v>784333.8800000036</v>
+        <v>774688.4900000008</v>
       </c>
       <c r="J20">
-        <v>-0.28723154977692195</v>
+        <v>-0.29599685987942465</v>
       </c>
       <c r="K20">
-        <v>-0.2873312312688218</v>
+        <v>-0.2976466708128013</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
         <v>370.47287369398555</v>
       </c>
       <c r="E21">
-        <v>377.68</v>
+        <v>378.92</v>
       </c>
       <c r="F21">
         <v>370.47</v>
@@ -2023,16 +2023,16 @@
         <v>806421.4786093751</v>
       </c>
       <c r="H21">
-        <v>582757.56</v>
+        <v>585609.9900000008</v>
       </c>
       <c r="I21">
-        <v>586335.2300000011</v>
+        <v>583783.6399999957</v>
       </c>
       <c r="J21">
-        <v>-0.27291714624082103</v>
+        <v>-0.2760812360718676</v>
       </c>
       <c r="K21">
-        <v>-0.2773536228165325</v>
+        <v>-0.2738164774457028</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -2080,7 +2080,7 @@
         <v>0.7904747724533081</v>
       </c>
       <c r="X21">
-        <v>0.801526068218561</v>
+        <v>0.8012858745341871</v>
       </c>
       <c r="Y21">
         <v>0.719028651714325</v>
@@ -2109,7 +2109,7 @@
         <v>236.53398952913864</v>
       </c>
       <c r="E22">
-        <v>240.14</v>
+        <v>240.08</v>
       </c>
       <c r="F22">
         <v>236.53</v>
@@ -2118,16 +2118,16 @@
         <v>559592.7028125001</v>
       </c>
       <c r="H22">
-        <v>367614.83000000066</v>
+        <v>367147.78999999986</v>
       </c>
       <c r="I22">
-        <v>366588.2300000012</v>
+        <v>365063.8899999982</v>
       </c>
       <c r="J22">
-        <v>-0.34490169697078393</v>
+        <v>-0.34762571390728386</v>
       </c>
       <c r="K22">
-        <v>-0.3430671483877882</v>
+        <v>-0.34390175541117046</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -2175,7 +2175,7 @@
         <v>0.8522438108921051</v>
       </c>
       <c r="X22">
-        <v>0.8521502356645682</v>
+        <v>0.8521497417596996</v>
       </c>
       <c r="Y22">
         <v>0.7339749336242676</v>
@@ -2204,7 +2204,7 @@
         <v>366.5435176578728</v>
       </c>
       <c r="E23">
-        <v>367.69</v>
+        <v>353.95</v>
       </c>
       <c r="F23">
         <v>366.54</v>
@@ -2213,16 +2213,16 @@
         <v>890316.30021875</v>
       </c>
       <c r="H23">
-        <v>539951.5100000006</v>
+        <v>552144.8299999984</v>
       </c>
       <c r="I23">
-        <v>550439.9700000006</v>
+        <v>559612.5899999994</v>
       </c>
       <c r="J23">
-        <v>-0.38174784639486226</v>
+        <v>-0.37144519328411374</v>
       </c>
       <c r="K23">
-        <v>-0.3935284461630828</v>
+        <v>-0.3798329539015102</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -2270,7 +2270,7 @@
         <v>0.6310444076855978</v>
       </c>
       <c r="X23">
-        <v>0.6109359084130974</v>
+        <v>0.6104917986502413</v>
       </c>
       <c r="Y23">
         <v>0.4843061566352844</v>
@@ -2299,7 +2299,7 @@
         <v>234.33676148704424</v>
       </c>
       <c r="E24">
-        <v>237.49</v>
+        <v>237.42</v>
       </c>
       <c r="F24">
         <v>234.34</v>
@@ -2308,16 +2308,16 @@
         <v>533411.51046875</v>
       </c>
       <c r="H24">
-        <v>360033.9999999998</v>
+        <v>341837.6299999988</v>
       </c>
       <c r="I24">
-        <v>365907.7299999989</v>
+        <v>360824.8199999993</v>
       </c>
       <c r="J24">
-        <v>-0.31402355813722993</v>
+        <v>-0.32355261759740694</v>
       </c>
       <c r="K24">
-        <v>-0.3250351877791125</v>
+        <v>-0.3591483811446072</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         <v>0.9972227513790131</v>
       </c>
       <c r="X24">
-        <v>0.997224778035883</v>
+        <v>0.9972245177071134</v>
       </c>
       <c r="Y24">
         <v>0.9952940344810486</v>
@@ -2394,7 +2394,7 @@
         <v>369.2005635828266</v>
       </c>
       <c r="E25">
-        <v>367.51</v>
+        <v>365.93</v>
       </c>
       <c r="F25">
         <v>369.2</v>
@@ -2403,16 +2403,16 @@
         <v>895263.256078125</v>
       </c>
       <c r="H25">
-        <v>543706.2000000003</v>
+        <v>599196.269999998</v>
       </c>
       <c r="I25">
-        <v>582552.090000001</v>
+        <v>579893.3600000005</v>
       </c>
       <c r="J25">
-        <v>-0.3492952089288419</v>
+        <v>-0.35226498344147816</v>
       </c>
       <c r="K25">
-        <v>-0.3926856750696871</v>
+        <v>-0.33070382825171</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         <v>0.7484132647514343</v>
       </c>
       <c r="X25">
-        <v>0.6981701350214314</v>
+        <v>0.6982920345600719</v>
       </c>
       <c r="Y25">
         <v>0.6164996027946472</v>
@@ -2489,7 +2489,7 @@
         <v>239.06366887064294</v>
       </c>
       <c r="E26">
-        <v>244.91</v>
+        <v>244.86</v>
       </c>
       <c r="F26">
         <v>239.06</v>
@@ -2498,16 +2498,16 @@
         <v>588706.8608437501</v>
       </c>
       <c r="H26">
-        <v>395414.7900000012</v>
+        <v>383320.7799999999</v>
       </c>
       <c r="I26">
-        <v>393658.0000000021</v>
+        <v>385178.6000000005</v>
       </c>
       <c r="J26">
-        <v>-0.331317458342848</v>
+        <v>-0.3457208916370493</v>
       </c>
       <c r="K26">
-        <v>-0.3283333076273608</v>
+        <v>-0.3488766557763323</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -2555,7 +2555,7 @@
         <v>0.9933198392391205</v>
       </c>
       <c r="X26">
-        <v>0.9933143407200014</v>
+        <v>0.9933159852928636</v>
       </c>
       <c r="Y26">
         <v>0.9876328706741333</v>
@@ -2584,7 +2584,7 @@
         <v>371.1067151006221</v>
       </c>
       <c r="E27">
-        <v>374.3</v>
+        <v>375.56</v>
       </c>
       <c r="F27">
         <v>371.11</v>
@@ -2593,16 +2593,16 @@
         <v>850291.7773125</v>
       </c>
       <c r="H27">
-        <v>619176.9500000001</v>
+        <v>622913.0799999997</v>
       </c>
       <c r="I27">
-        <v>609268.8900000011</v>
+        <v>610245.8899999986</v>
       </c>
       <c r="J27">
-        <v>-0.2834590357609892</v>
+        <v>-0.282310018416513</v>
       </c>
       <c r="K27">
-        <v>-0.27180649452236255</v>
+        <v>-0.2674125557595906</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
         <v>0.813204437494278</v>
       </c>
       <c r="X27">
-        <v>0.8330670060034264</v>
+        <v>0.8325922973661882</v>
       </c>
       <c r="Y27">
         <v>0.6857811808586121</v>
@@ -2679,7 +2679,7 @@
         <v>370.7444376004047</v>
       </c>
       <c r="E28">
-        <v>371.19</v>
+        <v>361.5</v>
       </c>
       <c r="F28">
         <v>370.74</v>
@@ -2688,16 +2688,16 @@
         <v>893793.9065</v>
       </c>
       <c r="H28">
-        <v>593374.3999999996</v>
+        <v>615661.1600000015</v>
       </c>
       <c r="I28">
-        <v>594756.2800000008</v>
+        <v>594120.3699999994</v>
       </c>
       <c r="J28">
-        <v>-0.3345711179336611</v>
+        <v>-0.33528259067405114</v>
       </c>
       <c r="K28">
-        <v>-0.33611720142108675</v>
+        <v>-0.31118219141718717</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>0.7062302728494009</v>
       </c>
       <c r="X28">
-        <v>0.7655380594806622</v>
+        <v>0.7662099909840393</v>
       </c>
       <c r="Y28">
         <v>0.4379631578922272</v>
@@ -2774,7 +2774,7 @@
         <v>237.23200376810422</v>
       </c>
       <c r="E29">
-        <v>242.52</v>
+        <v>242.29</v>
       </c>
       <c r="F29">
         <v>237.23</v>
@@ -2783,16 +2783,16 @@
         <v>584574.7331875</v>
       </c>
       <c r="H29">
-        <v>406187.7499999999</v>
+        <v>390146.7200000012</v>
       </c>
       <c r="I29">
-        <v>356633.54000000097</v>
+        <v>368737.5500000007</v>
       </c>
       <c r="J29">
-        <v>-0.38992652307192316</v>
+        <v>-0.3692208556647802</v>
       </c>
       <c r="K29">
-        <v>-0.30515684832085144</v>
+        <v>-0.332597360353474</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
         <v>0.8294468224048615</v>
       </c>
       <c r="X29">
-        <v>0.8296518009049669</v>
+        <v>0.8297632859597448</v>
       </c>
       <c r="Y29">
         <v>0.7087990045547485</v>
@@ -2869,7 +2869,7 @@
         <v>372.25901245316396</v>
       </c>
       <c r="E30">
-        <v>376.79</v>
+        <v>377.37</v>
       </c>
       <c r="F30">
         <v>372.26</v>
@@ -2878,16 +2878,16 @@
         <v>897705.558875</v>
       </c>
       <c r="H30">
-        <v>597127.5499999996</v>
+        <v>585491.27</v>
       </c>
       <c r="I30">
-        <v>588688.6000000001</v>
+        <v>588211.7799999994</v>
       </c>
       <c r="J30">
-        <v>-0.3442297486296714</v>
+        <v>-0.34476090274282867</v>
       </c>
       <c r="K30">
-        <v>-0.3348291718853599</v>
+        <v>-0.3477914175626419</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
         <v>0.9016911089420319</v>
       </c>
       <c r="X30">
-        <v>0.9064905634024182</v>
+        <v>0.9064373687873619</v>
       </c>
       <c r="Y30">
         <v>0.8705822825431824</v>
@@ -2964,7 +2964,7 @@
         <v>235.89975493456654</v>
       </c>
       <c r="E31">
-        <v>239.93</v>
+        <v>239.82</v>
       </c>
       <c r="F31">
         <v>235.9</v>
@@ -2973,16 +2973,16 @@
         <v>572696.5886875</v>
       </c>
       <c r="H31">
-        <v>403176.09999999974</v>
+        <v>399103.7399999988</v>
       </c>
       <c r="I31">
-        <v>402532.75999999995</v>
+        <v>403003.79000000004</v>
       </c>
       <c r="J31">
-        <v>-0.29712736560467334</v>
+        <v>-0.2963048882068603</v>
       </c>
       <c r="K31">
-        <v>-0.2960040133572395</v>
+        <v>-0.3031148641645298</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -3030,7 +3030,7 @@
         <v>0.9866441488265991</v>
       </c>
       <c r="X31">
-        <v>0.9866730437575632</v>
+        <v>0.9866718508720423</v>
       </c>
       <c r="Y31">
         <v>0.9758704900741577</v>
@@ -3059,7 +3059,7 @@
         <v>372.87641404951376</v>
       </c>
       <c r="E32">
-        <v>379.27</v>
+        <v>379.2</v>
       </c>
       <c r="F32">
         <v>372.88</v>
@@ -3068,16 +3068,16 @@
         <v>858762.7599375</v>
       </c>
       <c r="H32">
-        <v>581726.9200000005</v>
+        <v>580241.9800000004</v>
       </c>
       <c r="I32">
-        <v>634476.1899999996</v>
+        <v>631138.9999999993</v>
       </c>
       <c r="J32">
-        <v>-0.26117407554307986</v>
+        <v>-0.26506011969367066</v>
       </c>
       <c r="K32">
-        <v>-0.3225988047707867</v>
+        <v>-0.32432796685055376</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
         <v>238.60140604129373</v>
       </c>
       <c r="E33">
-        <v>243.47</v>
+        <v>243.5</v>
       </c>
       <c r="F33">
         <v>238.6</v>
@@ -3163,16 +3163,16 @@
         <v>586904.6228125</v>
       </c>
       <c r="H33">
-        <v>397755.0000000008</v>
+        <v>399727.50000000006</v>
       </c>
       <c r="I33">
-        <v>400110.34000000067</v>
+        <v>400855.539999999</v>
       </c>
       <c r="J33">
-        <v>-0.3182702530393512</v>
+        <v>-0.31700054077089557</v>
       </c>
       <c r="K33">
-        <v>-0.322283409365694</v>
+        <v>-0.3189225566422194</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -3220,7 +3220,7 @@
         <v>0.9899944961071014</v>
       </c>
       <c r="X33">
-        <v>0.9899965978240969</v>
+        <v>0.9899969336948173</v>
       </c>
       <c r="Y33">
         <v>0.9830652475357056</v>
@@ -3249,7 +3249,7 @@
         <v>369.61348279181516</v>
       </c>
       <c r="E34">
-        <v>379.78</v>
+        <v>379.34</v>
       </c>
       <c r="F34">
         <v>369.61</v>
@@ -3258,16 +3258,16 @@
         <v>898239.93771875</v>
       </c>
       <c r="H34">
-        <v>630150.38</v>
+        <v>633009.3300000009</v>
       </c>
       <c r="I34">
-        <v>625517.9499999981</v>
+        <v>625139.3299999986</v>
       </c>
       <c r="J34">
-        <v>-0.30361819405556706</v>
+        <v>-0.30403970726612534</v>
       </c>
       <c r="K34">
-        <v>-0.29846096400435507</v>
+        <v>-0.2952781284612576</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3315,7 +3315,7 @@
         <v>0.7704202234745026</v>
       </c>
       <c r="X34">
-        <v>0.7741709593541907</v>
+        <v>0.7741062814860232</v>
       </c>
       <c r="Y34">
         <v>0.5520116090774536</v>
@@ -3353,16 +3353,16 @@
         <v>5424386.1137500005</v>
       </c>
       <c r="H35">
-        <v>3411092.7000000007</v>
+        <v>3200045.879999998</v>
       </c>
       <c r="I35">
-        <v>3412434.8700000052</v>
+        <v>3201373.469999997</v>
       </c>
       <c r="J35">
-        <v>-0.3709085602608565</v>
+        <v>-0.4098182904264506</v>
       </c>
       <c r="K35">
-        <v>-0.3711559928683183</v>
+        <v>-0.4100630351721526</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -3424,7 +3424,7 @@
         <v>124.26560305683645</v>
       </c>
       <c r="E36">
-        <v>126.24</v>
+        <v>126.23</v>
       </c>
       <c r="F36">
         <v>124.23</v>
@@ -3433,16 +3433,16 @@
         <v>264982.38575</v>
       </c>
       <c r="H36">
-        <v>225453.62999999936</v>
+        <v>225095.98000000042</v>
       </c>
       <c r="I36">
-        <v>210540.3000000003</v>
+        <v>209885.7900000009</v>
       </c>
       <c r="J36">
-        <v>-0.20545548941265696</v>
+        <v>-0.20792550264824197</v>
       </c>
       <c r="K36">
-        <v>-0.1491750315332069</v>
+        <v>-0.15052474388856465</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -3519,7 +3519,7 @@
         <v>123.18186977450087</v>
       </c>
       <c r="E37">
-        <v>125.03</v>
+        <v>118.92</v>
       </c>
       <c r="F37">
         <v>123.17</v>
@@ -3528,16 +3528,16 @@
         <v>277058.5811875</v>
       </c>
       <c r="H37">
-        <v>181634.44999999987</v>
+        <v>187695.16000000018</v>
       </c>
       <c r="I37">
-        <v>185055.21000000034</v>
+        <v>186577.86000000045</v>
       </c>
       <c r="J37">
-        <v>-0.33207190621262933</v>
+        <v>-0.32657613707429806</v>
       </c>
       <c r="K37">
-        <v>-0.34441860915660155</v>
+        <v>-0.32254341592481817</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -3585,7 +3585,7 @@
         <v>0.7779085437456766</v>
       </c>
       <c r="X37">
-        <v>0.7575092045177529</v>
+        <v>0.7563747943315283</v>
       </c>
       <c r="Y37">
         <v>0.6722833514213562</v>
@@ -3623,16 +3623,16 @@
         <v>279505.0353125</v>
       </c>
       <c r="H38">
-        <v>206213.97000000012</v>
+        <v>194853.31999999986</v>
       </c>
       <c r="I38">
-        <v>208929.51000000114</v>
+        <v>204550.3600000006</v>
       </c>
       <c r="J38">
-        <v>-0.25250180281579565</v>
+        <v>-0.2681693202009635</v>
       </c>
       <c r="K38">
-        <v>-0.26221733440528894</v>
+        <v>-0.3028629348943767</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -3680,7 +3680,7 @@
         <v>0.6666513085365295</v>
       </c>
       <c r="X38">
-        <v>0.6666460422440421</v>
+        <v>0.6666481890444158</v>
       </c>
       <c r="Y38">
         <v>0.6264314651489258</v>
@@ -3718,16 +3718,16 @@
         <v>247551.24514062502</v>
       </c>
       <c r="H39">
-        <v>210503.4900000006</v>
+        <v>205361.2900000006</v>
       </c>
       <c r="I39">
-        <v>210232.2200000003</v>
+        <v>205060.4400000001</v>
       </c>
       <c r="J39">
-        <v>-0.15075272644831628</v>
+        <v>-0.17164448159607285</v>
       </c>
       <c r="K39">
-        <v>-0.1496569129336389</v>
+        <v>-0.17042917767049737</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         <v>121.72871093484056</v>
       </c>
       <c r="E40">
-        <v>126.23</v>
+        <v>126.3</v>
       </c>
       <c r="F40">
         <v>121.73</v>
@@ -3798,16 +3798,16 @@
         <v>235608.508375</v>
       </c>
       <c r="H40">
-        <v>187501.68000000023</v>
+        <v>183193.42000000013</v>
       </c>
       <c r="I40">
-        <v>175662.0400000003</v>
+        <v>180226.14000000025</v>
       </c>
       <c r="J40">
-        <v>-0.25443252787623233</v>
+        <v>-0.23506098636663786</v>
       </c>
       <c r="K40">
-        <v>-0.2041812017180289</v>
+        <v>-0.2224668741231314</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -3855,7 +3855,7 @@
         <v>0.9834159016609192</v>
       </c>
       <c r="X40">
-        <v>0.9834990528412552</v>
+        <v>0.9834923695480506</v>
       </c>
       <c r="Y40">
         <v>0.967885434627533</v>
@@ -3884,7 +3884,7 @@
         <v>120.87717554136132</v>
       </c>
       <c r="E41">
-        <v>123.74</v>
+        <v>123.73</v>
       </c>
       <c r="F41">
         <v>120.88</v>
@@ -3893,16 +3893,16 @@
         <v>269707.395125</v>
       </c>
       <c r="H41">
-        <v>204377.80999999947</v>
+        <v>201729.69000000035</v>
       </c>
       <c r="I41">
-        <v>198508.96000000017</v>
+        <v>195452.50999999986</v>
       </c>
       <c r="J41">
-        <v>-0.2639839930677534</v>
+        <v>-0.27531645949339123</v>
       </c>
       <c r="K41">
-        <v>-0.2422239297321548</v>
+        <v>-0.2520424220978232</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3950,7 +3950,7 @@
         <v>0.9046740233898163</v>
       </c>
       <c r="X41">
-        <v>0.9050082442125046</v>
+        <v>0.9050305003761419</v>
       </c>
       <c r="Y41">
         <v>0.8122680187225342</v>
@@ -3979,7 +3979,7 @@
         <v>120.0414937883839</v>
       </c>
       <c r="E42">
-        <v>122.3</v>
+        <v>122.33</v>
       </c>
       <c r="F42">
         <v>120.04</v>
@@ -3988,16 +3988,16 @@
         <v>270018.56453125</v>
       </c>
       <c r="H42">
-        <v>205338.3100000007</v>
+        <v>205258.13999999987</v>
       </c>
       <c r="I42">
-        <v>204199.00000000052</v>
+        <v>201231.05999999953</v>
       </c>
       <c r="J42">
-        <v>-0.24375940463764662</v>
+        <v>-0.2547510192518244</v>
       </c>
       <c r="K42">
-        <v>-0.2395400280848603</v>
+        <v>-0.23983693359630173</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -4045,7 +4045,7 @@
         <v>0.8856760263442993</v>
       </c>
       <c r="X42">
-        <v>0.8858963498418937</v>
+        <v>0.885886133832419</v>
       </c>
       <c r="Y42">
         <v>0.778390109539032</v>
@@ -4083,16 +4083,16 @@
         <v>276318.81809375</v>
       </c>
       <c r="H43">
-        <v>206467.07000000007</v>
+        <v>206609.0600000001</v>
       </c>
       <c r="I43">
-        <v>205750.07000000015</v>
+        <v>196982.4899999998</v>
       </c>
       <c r="J43">
-        <v>-0.25538886052200443</v>
+        <v>-0.2871188022628007</v>
       </c>
       <c r="K43">
-        <v>-0.2527940318203391</v>
+        <v>-0.25228016888121824</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -4140,7 +4140,7 @@
         <v>0.9297216236591339</v>
       </c>
       <c r="X43">
-        <v>0.9297205351581003</v>
+        <v>0.9297251337711753</v>
       </c>
       <c r="Y43">
         <v>0.921430230140686</v>
@@ -4169,7 +4169,7 @@
         <v>125.47070361249024</v>
       </c>
       <c r="E44">
-        <v>127.4</v>
+        <v>127.39</v>
       </c>
       <c r="F44">
         <v>125.48</v>
@@ -4178,16 +4178,16 @@
         <v>275909.47353125</v>
       </c>
       <c r="H44">
-        <v>216238.72000000006</v>
+        <v>216368.73999999883</v>
       </c>
       <c r="I44">
-        <v>215600.3699999995</v>
+        <v>212705.16999999955</v>
       </c>
       <c r="J44">
-        <v>-0.21858293866962783</v>
+        <v>-0.22907623548523007</v>
       </c>
       <c r="K44">
-        <v>-0.21626931749587622</v>
+        <v>-0.21579807597475448</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -4235,7 +4235,7 @@
         <v>0.851101279258728</v>
       </c>
       <c r="X44">
-        <v>0.8510582489557049</v>
+        <v>0.8510361973543399</v>
       </c>
       <c r="Y44">
         <v>0.7123515605926514</v>
@@ -4264,7 +4264,7 @@
         <v>116.75256223313664</v>
       </c>
       <c r="E45">
-        <v>118.57</v>
+        <v>118.52</v>
       </c>
       <c r="F45">
         <v>116.75</v>
@@ -4273,16 +4273,16 @@
         <v>279143.835625</v>
       </c>
       <c r="H45">
-        <v>201668.6000000004</v>
+        <v>201636.1499999996</v>
       </c>
       <c r="I45">
-        <v>199929.34999999977</v>
+        <v>191503.72000000023</v>
       </c>
       <c r="J45">
-        <v>-0.28377658939750494</v>
+        <v>-0.313960419110723</v>
       </c>
       <c r="K45">
-        <v>-0.2775459305828244</v>
+        <v>-0.2776621788959142</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -4330,7 +4330,7 @@
         <v>0.8419512808322906</v>
       </c>
       <c r="X45">
-        <v>0.8418828661570861</v>
+        <v>0.8419988040296486</v>
       </c>
       <c r="Y45">
         <v>0.7161607146263123</v>
@@ -4359,7 +4359,7 @@
         <v>124.10312756987287</v>
       </c>
       <c r="E46">
-        <v>125.9</v>
+        <v>126.07</v>
       </c>
       <c r="F46">
         <v>124.1</v>
@@ -4368,16 +4368,16 @@
         <v>291034.884875</v>
       </c>
       <c r="H46">
-        <v>214372.36999999982</v>
+        <v>214090.04999999984</v>
       </c>
       <c r="I46">
-        <v>214446.27999999915</v>
+        <v>204540.21000000063</v>
       </c>
       <c r="J46">
-        <v>-0.26315953466504804</v>
+        <v>-0.29719693194906505</v>
       </c>
       <c r="K46">
-        <v>-0.26341349047529766</v>
+        <v>-0.2643835460070297</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -4425,7 +4425,7 @@
         <v>0.7650662958621979</v>
       </c>
       <c r="X46">
-        <v>0.7650008274414574</v>
+        <v>0.7650227528826635</v>
       </c>
       <c r="Y46">
         <v>0.6473265886306763</v>
@@ -4454,7 +4454,7 @@
         <v>130.9085264508188</v>
       </c>
       <c r="E47">
-        <v>132.72</v>
+        <v>132.74</v>
       </c>
       <c r="F47">
         <v>130.92</v>
@@ -4463,16 +4463,16 @@
         <v>292941.29778125003</v>
       </c>
       <c r="H47">
-        <v>224439.10000000018</v>
+        <v>224158.8599999998</v>
       </c>
       <c r="I47">
-        <v>223754.9800000001</v>
+        <v>222105.34000000014</v>
       </c>
       <c r="J47">
-        <v>-0.23617809542481746</v>
+        <v>-0.2418093942976442</v>
       </c>
       <c r="K47">
-        <v>-0.23384274699432425</v>
+        <v>-0.23479938916844897</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -4520,7 +4520,7 @@
         <v>0.8466036021709442</v>
       </c>
       <c r="X47">
-        <v>0.8466980929066061</v>
+        <v>0.8467186372341261</v>
       </c>
       <c r="Y47">
         <v>0.7241121530532837</v>
@@ -4549,7 +4549,7 @@
         <v>118.41081365152584</v>
       </c>
       <c r="E48">
-        <v>121.09</v>
+        <v>121.1</v>
       </c>
       <c r="F48">
         <v>118.44</v>
@@ -4558,16 +4558,16 @@
         <v>281187.1920625</v>
       </c>
       <c r="H48">
-        <v>205150.85999999952</v>
+        <v>204871.91999999934</v>
       </c>
       <c r="I48">
-        <v>200779.8799999999</v>
+        <v>194845.4799999999</v>
       </c>
       <c r="J48">
-        <v>-0.285956524095976</v>
+        <v>-0.3070613260482674</v>
       </c>
       <c r="K48">
-        <v>-0.2704117904687484</v>
+        <v>-0.27140379866782094</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -4615,7 +4615,7 @@
         <v>0.8725321888923645</v>
       </c>
       <c r="X48">
-        <v>0.8730019373729163</v>
+        <v>0.8729970640357773</v>
       </c>
       <c r="Y48">
         <v>0.762785792350769</v>
@@ -4644,7 +4644,7 @@
         <v>112.27774131099156</v>
       </c>
       <c r="E49">
-        <v>113.83</v>
+        <v>113.84</v>
       </c>
       <c r="F49">
         <v>112.23</v>
@@ -4653,16 +4653,16 @@
         <v>215944.514375</v>
       </c>
       <c r="H49">
-        <v>176188.7200000002</v>
+        <v>176128.15000000055</v>
       </c>
       <c r="I49">
-        <v>193890.17000000048</v>
+        <v>193873.80000000002</v>
       </c>
       <c r="J49">
-        <v>-0.10212968103788407</v>
+        <v>-0.10220548754793986</v>
       </c>
       <c r="K49">
-        <v>-0.18410189529501816</v>
+        <v>-0.18438238401303428</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -4748,16 +4748,16 @@
         <v>135464.283875</v>
       </c>
       <c r="H50">
-        <v>98060.66000000016</v>
+        <v>98216.92000000023</v>
       </c>
       <c r="I50">
-        <v>98379.99999999993</v>
+        <v>98310.66000000006</v>
       </c>
       <c r="J50">
-        <v>-0.2737569107826214</v>
+        <v>-0.2742687800223676</v>
       </c>
       <c r="K50">
-        <v>-0.2761142849248302</v>
+        <v>-0.27496077054059403</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -4819,7 +4819,7 @@
         <v>110.62788457108744</v>
       </c>
       <c r="E51">
-        <v>112.3</v>
+        <v>112.31</v>
       </c>
       <c r="F51">
         <v>110.6</v>
@@ -4828,16 +4828,16 @@
         <v>253369.3274375</v>
       </c>
       <c r="H51">
-        <v>191601.66000000056</v>
+        <v>191814.4800000007</v>
       </c>
       <c r="I51">
-        <v>191129.89000000016</v>
+        <v>191308.27999999974</v>
       </c>
       <c r="J51">
-        <v>-0.24564708785775494</v>
+        <v>-0.2449430168409363</v>
       </c>
       <c r="K51">
-        <v>-0.24378510241235105</v>
+        <v>-0.24294514280811425</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4885,7 +4885,7 @@
         <v>0.9626638889312744</v>
       </c>
       <c r="X51">
-        <v>0.9626838051242314</v>
+        <v>0.9626904525182852</v>
       </c>
       <c r="Y51">
         <v>0.9442288279533386</v>
@@ -4914,7 +4914,7 @@
         <v>58.5967501938149</v>
       </c>
       <c r="E52">
-        <v>61.21</v>
+        <v>59.74</v>
       </c>
       <c r="F52">
         <v>58.6</v>
@@ -4923,16 +4923,16 @@
         <v>119194.47425</v>
       </c>
       <c r="H52">
-        <v>106030.69000000006</v>
+        <v>103521.44999999987</v>
       </c>
       <c r="I52">
-        <v>100388.20999999973</v>
+        <v>100198.83000000006</v>
       </c>
       <c r="J52">
-        <v>-0.1577779873465927</v>
+        <v>-0.15936681938928002</v>
       </c>
       <c r="K52">
-        <v>-0.11043955126971784</v>
+        <v>-0.13149119830108344</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -4980,7 +4980,7 @@
         <v>0.9952588081359863</v>
       </c>
       <c r="X52">
-        <v>0.9945255588123589</v>
+        <v>0.9944092583263212</v>
       </c>
       <c r="Y52">
         <v>0.991319477558136</v>
@@ -5009,7 +5009,7 @@
         <v>119.07112961905189</v>
       </c>
       <c r="E53">
-        <v>122.2</v>
+        <v>122.07</v>
       </c>
       <c r="F53">
         <v>119.05</v>
@@ -5018,16 +5018,16 @@
         <v>267140.7060625</v>
       </c>
       <c r="H53">
-        <v>206125.56000000035</v>
+        <v>205241.84999999934</v>
       </c>
       <c r="I53">
-        <v>205752.11000000034</v>
+        <v>201652.92000000027</v>
       </c>
       <c r="J53">
-        <v>-0.22979873403545342</v>
+        <v>-0.24514341909083026</v>
       </c>
       <c r="K53">
-        <v>-0.22840078160242872</v>
+        <v>-0.23170881358687012</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -5075,7 +5075,7 @@
         <v>0.843268871307373</v>
       </c>
       <c r="X53">
-        <v>0.8438735427448264</v>
+        <v>0.8439802614170354</v>
       </c>
       <c r="Y53">
         <v>0.6907517313957214</v>
@@ -5104,7 +5104,7 @@
         <v>168.56033444445646</v>
       </c>
       <c r="E54">
-        <v>175.18</v>
+        <v>173.03</v>
       </c>
       <c r="F54">
         <v>150.52</v>
@@ -5113,16 +5113,16 @@
         <v>361110.8783125</v>
       </c>
       <c r="H54">
-        <v>298728.4899999997</v>
+        <v>293516.919999999</v>
       </c>
       <c r="I54">
-        <v>260199.59999999995</v>
+        <v>260009.5299999995</v>
       </c>
       <c r="J54">
-        <v>-0.27944679701721126</v>
+        <v>-0.2799731450488426</v>
       </c>
       <c r="K54">
-        <v>-0.17275134054121605</v>
+        <v>-0.18718338984517163</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -5170,7 +5170,7 @@
         <v>0.9855310320854187</v>
       </c>
       <c r="X54">
-        <v>0.9856488374403087</v>
+        <v>0.9856804824481136</v>
       </c>
       <c r="Y54">
         <v>0.9830591678619385</v>
@@ -5199,7 +5199,7 @@
         <v>56.743204455406456</v>
       </c>
       <c r="E55">
-        <v>58.18</v>
+        <v>57.36</v>
       </c>
       <c r="F55">
         <v>56.74</v>
@@ -5208,16 +5208,16 @@
         <v>111803.671671875</v>
       </c>
       <c r="H55">
-        <v>101661.64999999989</v>
+        <v>100718.25</v>
       </c>
       <c r="I55">
-        <v>96835.46000000015</v>
+        <v>97126.8999999999</v>
       </c>
       <c r="J55">
-        <v>-0.1338794285379467</v>
+        <v>-0.13127271629279716</v>
       </c>
       <c r="K55">
-        <v>-0.09071277821394126</v>
+        <v>-0.0991507837453572</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -5265,7 +5265,7 @@
         <v>0.7142086029052734</v>
       </c>
       <c r="X55">
-        <v>0.6614543163205797</v>
+        <v>0.6566702240503706</v>
       </c>
       <c r="Y55">
         <v>0.4353100657463074</v>
@@ -5303,16 +5303,16 @@
         <v>103219.02082812501</v>
       </c>
       <c r="H56">
-        <v>96140.8800000004</v>
+        <v>95509.22000000013</v>
       </c>
       <c r="I56">
-        <v>95933.09000000003</v>
+        <v>96042.63999999984</v>
       </c>
       <c r="J56">
-        <v>-0.07058709499150491</v>
+        <v>-0.06952575959885252</v>
       </c>
       <c r="K56">
-        <v>-0.06857399703404246</v>
+        <v>-0.0746936055609638</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5374,7 +5374,7 @@
         <v>168.7324221607141</v>
       </c>
       <c r="E57">
-        <v>171.57</v>
+        <v>171.66</v>
       </c>
       <c r="F57">
         <v>168.73</v>
@@ -5383,16 +5383,16 @@
         <v>380573.5991171875</v>
       </c>
       <c r="H57">
-        <v>279210.8800000001</v>
+        <v>280203.1399999998</v>
       </c>
       <c r="I57">
-        <v>288784.7199999997</v>
+        <v>288563.15000000043</v>
       </c>
       <c r="J57">
-        <v>-0.24118561910261113</v>
+        <v>-0.24176781923555055</v>
       </c>
       <c r="K57">
-        <v>-0.26634196211276184</v>
+        <v>-0.26373468719326826</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -5440,7 +5440,7 @@
         <v>0.5803835690021515</v>
       </c>
       <c r="X57">
-        <v>0.6315674323779735</v>
+        <v>0.6315267567562867</v>
       </c>
       <c r="Y57">
         <v>0.4520184397697449</v>
@@ -5478,16 +5478,16 @@
         <v>376216.25653125</v>
       </c>
       <c r="H58">
-        <v>291866.9499999996</v>
+        <v>292049.4700000001</v>
       </c>
       <c r="I58">
-        <v>291818.6400000003</v>
+        <v>291761.80999999976</v>
       </c>
       <c r="J58">
-        <v>-0.22433272105092916</v>
+        <v>-0.22448377778761705</v>
       </c>
       <c r="K58">
-        <v>-0.22420431086354192</v>
+        <v>-0.22371916436380443</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -5549,7 +5549,7 @@
         <v>111.8848157134316</v>
       </c>
       <c r="E59">
-        <v>115.02</v>
+        <v>114.97</v>
       </c>
       <c r="F59">
         <v>111.85</v>
@@ -5558,16 +5558,16 @@
         <v>259544.44775</v>
       </c>
       <c r="H59">
-        <v>194989.27999999994</v>
+        <v>194907.94999999987</v>
       </c>
       <c r="I59">
-        <v>193298.7399999995</v>
+        <v>193358.7100000005</v>
       </c>
       <c r="J59">
-        <v>-0.2552383929777226</v>
+        <v>-0.25500733428808053</v>
       </c>
       <c r="K59">
-        <v>-0.24872490361335442</v>
+        <v>-0.24903826034552545</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5615,7 +5615,7 @@
         <v>0.9448669254779816</v>
       </c>
       <c r="X59">
-        <v>0.9448813437381243</v>
+        <v>0.9448702388205317</v>
       </c>
       <c r="Y59">
         <v>0.8904971480369568</v>
@@ -5644,7 +5644,7 @@
         <v>109.86903584095278</v>
       </c>
       <c r="E60">
-        <v>110.58</v>
+        <v>110.54</v>
       </c>
       <c r="F60">
         <v>109.87</v>
@@ -5653,16 +5653,16 @@
         <v>272527.6270625</v>
       </c>
       <c r="H60">
-        <v>189821.53000000035</v>
+        <v>189193.36999999956</v>
       </c>
       <c r="I60">
-        <v>190048.94000000064</v>
+        <v>189924.7399999998</v>
       </c>
       <c r="J60">
-        <v>-0.30264339785112554</v>
+        <v>-0.30309913146367545</v>
       </c>
       <c r="K60">
-        <v>-0.30347784536182926</v>
+        <v>-0.3057827859903136</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -5710,7 +5710,7 @@
         <v>0.9668639302253723</v>
       </c>
       <c r="X60">
-        <v>0.9668767547494551</v>
+        <v>0.9668732639135708</v>
       </c>
       <c r="Y60">
         <v>0.9546698927879333</v>
@@ -5739,7 +5739,7 @@
         <v>451.4562124773123</v>
       </c>
       <c r="E61">
-        <v>451.33</v>
+        <v>451.37</v>
       </c>
       <c r="F61">
         <v>451.46</v>
@@ -5748,16 +5748,16 @@
         <v>910426.1154375001</v>
       </c>
       <c r="H61">
-        <v>782367.1599999971</v>
+        <v>778456.869999998</v>
       </c>
       <c r="I61">
-        <v>782867.660000003</v>
+        <v>781735.4600000015</v>
       </c>
       <c r="J61">
-        <v>-0.1401085198178873</v>
+        <v>-0.14135211331856076</v>
       </c>
       <c r="K61">
-        <v>-0.14065826239613627</v>
+        <v>-0.144953273197886</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5843,16 +5843,16 @@
         <v>1083195.76996875</v>
       </c>
       <c r="H62">
-        <v>883440.0500000028</v>
+        <v>880417.4399999998</v>
       </c>
       <c r="I62">
-        <v>884032.2200000017</v>
+        <v>878073.610000002</v>
       </c>
       <c r="J62">
-        <v>-0.18386662456639216</v>
+        <v>-0.18936757847075578</v>
       </c>
       <c r="K62">
-        <v>-0.1844133124472135</v>
+        <v>-0.18720376832213834</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5923,16 +5923,16 @@
         <v>1062625.4551796876</v>
       </c>
       <c r="H63">
-        <v>862444.2100000001</v>
+        <v>851145.6300000016</v>
       </c>
       <c r="I63">
-        <v>861089.1999999991</v>
+        <v>857294.1500000005</v>
       </c>
       <c r="J63">
-        <v>-0.18965878729642244</v>
+        <v>-0.19323017736759002</v>
       </c>
       <c r="K63">
-        <v>-0.18838363433128685</v>
+        <v>-0.19901633651710818</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -6003,16 +6003,16 @@
         <v>1044686.848125</v>
       </c>
       <c r="H64">
-        <v>802377.9799999996</v>
+        <v>804524.8799999984</v>
       </c>
       <c r="I64">
-        <v>803482.4600000002</v>
+        <v>804516.7299999979</v>
       </c>
       <c r="J64">
-        <v>-0.23088678541125748</v>
+        <v>-0.22989675667503476</v>
       </c>
       <c r="K64">
-        <v>-0.23194402088998767</v>
+        <v>-0.22988895529415673</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -6083,16 +6083,16 @@
         <v>2267763.24325</v>
       </c>
       <c r="H65">
-        <v>1368111.3999999997</v>
+        <v>1365289.2900000021</v>
       </c>
       <c r="I65">
-        <v>1369518.230000005</v>
+        <v>1365390.45</v>
       </c>
       <c r="J65">
-        <v>-0.3960929413260499</v>
+        <v>-0.3979131401551346</v>
       </c>
       <c r="K65">
-        <v>-0.3967133014999758</v>
+        <v>-0.39795774798635286</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -6163,16 +6163,16 @@
         <v>1913829.6795</v>
       </c>
       <c r="H66">
-        <v>1231509.7400000002</v>
+        <v>1230754.1199999969</v>
       </c>
       <c r="I66">
-        <v>1231365.3299999943</v>
+        <v>1232496.5000000007</v>
       </c>
       <c r="J66">
-        <v>-0.3565961782337412</v>
+        <v>-0.3560051277279815</v>
       </c>
       <c r="K66">
-        <v>-0.35652072219836206</v>
+        <v>-0.35691554312108953</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -6243,16 +6243,16 @@
         <v>34614.4205</v>
       </c>
       <c r="H67">
-        <v>26637.46000000004</v>
+        <v>26684.019999999968</v>
       </c>
       <c r="I67">
-        <v>26712.810000000052</v>
+        <v>26640.179999999957</v>
       </c>
       <c r="J67">
-        <v>-0.22827510574674933</v>
+        <v>-0.2303733641879125</v>
       </c>
       <c r="K67">
-        <v>-0.23045194415431455</v>
+        <v>-0.22910684002351078</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -6323,16 +6323,16 @@
         <v>20633.5035</v>
       </c>
       <c r="H68">
-        <v>17196.809999999998</v>
+        <v>17186.86000000001</v>
       </c>
       <c r="I68">
-        <v>17190.36999999997</v>
+        <v>17232.639999999934</v>
       </c>
       <c r="J68">
-        <v>-0.16687100666157006</v>
+        <v>-0.16482239673936447</v>
       </c>
       <c r="K68">
-        <v>-0.16655889291898496</v>
+        <v>-0.16704111834424956</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -6403,16 +6403,16 @@
         <v>1060573.5794375</v>
       </c>
       <c r="H69">
-        <v>849689.4400000012</v>
+        <v>848962.6199999995</v>
       </c>
       <c r="I69">
-        <v>849748.2200000014</v>
+        <v>849413.7800000021</v>
       </c>
       <c r="J69">
-        <v>-0.1987842838299959</v>
+        <v>-0.1990996226301352</v>
       </c>
       <c r="K69">
-        <v>-0.1988397066701833</v>
+        <v>-0.19952501508639633</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -6483,16 +6483,16 @@
         <v>129415.845</v>
       </c>
       <c r="H70">
-        <v>114440.9699999999</v>
+        <v>114531.87000000014</v>
       </c>
       <c r="I70">
-        <v>114410.4300000002</v>
+        <v>114381.82999999978</v>
       </c>
       <c r="J70">
-        <v>-0.11594727832592527</v>
+        <v>-0.11616827135811861</v>
       </c>
       <c r="K70">
-        <v>-0.11571129485728816</v>
+        <v>-0.11500890791231831</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -6563,16 +6563,16 @@
         <v>66440.65612500001</v>
       </c>
       <c r="H71">
-        <v>55365.099999999955</v>
+        <v>55380.380000000114</v>
       </c>
       <c r="I71">
-        <v>55411.01000000004</v>
+        <v>55433.85999999997</v>
       </c>
       <c r="J71">
-        <v>-0.16600748349397745</v>
+        <v>-0.16566356756459613</v>
       </c>
       <c r="K71">
-        <v>-0.16669847606806806</v>
+        <v>-0.16646849640062752</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6866,13 +6866,13 @@
         <v>6850.44</v>
       </c>
       <c r="D2">
-        <v>11750669.109999998</v>
+        <v>11748293.760000022</v>
       </c>
       <c r="E2">
         <v>6850.44</v>
       </c>
       <c r="F2">
-        <v>11749716.379999992</v>
+        <v>11746907.960000018</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -6906,13 +6906,13 @@
         <v>1693.19</v>
       </c>
       <c r="D3">
-        <v>2936828.719999997</v>
+        <v>2937445.209999999</v>
       </c>
       <c r="E3">
         <v>1693.19</v>
       </c>
       <c r="F3">
-        <v>2937236.7100000083</v>
+        <v>2937699.7800000003</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -6946,13 +6946,13 @@
         <v>2906.82</v>
       </c>
       <c r="D4">
-        <v>5046186.889999997</v>
+        <v>5045869.819999991</v>
       </c>
       <c r="E4">
         <v>2906.82</v>
       </c>
       <c r="F4">
-        <v>5045631.119999985</v>
+        <v>5045545.209999988</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -6986,13 +6986,13 @@
         <v>3104.91</v>
       </c>
       <c r="D5">
-        <v>5357884.150000015</v>
+        <v>5357584.599999997</v>
       </c>
       <c r="E5">
         <v>3104.91</v>
       </c>
       <c r="F5">
-        <v>5357553.279999997</v>
+        <v>5358992.709999977</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -7026,13 +7026,13 @@
         <v>930.44</v>
       </c>
       <c r="D6">
-        <v>1590331.260000006</v>
+        <v>1586904.020000001</v>
       </c>
       <c r="E6">
         <v>930.44</v>
       </c>
       <c r="F6">
-        <v>1589563.1200000024</v>
+        <v>1586967.599999998</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -7063,16 +7063,16 @@
         </is>
       </c>
       <c r="C7">
-        <v>872.5</v>
+        <v>872.62</v>
       </c>
       <c r="D7">
-        <v>1474814.5499999996</v>
+        <v>1470648.6999999953</v>
       </c>
       <c r="E7">
         <v>866.55</v>
       </c>
       <c r="F7">
-        <v>1479402.0700000008</v>
+        <v>1475226.4500000032</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -7097,7 +7097,7 @@
         <v>0.6519851982593536</v>
       </c>
       <c r="O7">
-        <v>0.6512579033929947</v>
+        <v>0.6512806921393035</v>
       </c>
       <c r="P7">
         <v>0.5486889481544495</v>
@@ -7118,16 +7118,16 @@
         </is>
       </c>
       <c r="C8">
-        <v>875.18</v>
+        <v>875.52</v>
       </c>
       <c r="D8">
-        <v>1427502.510000007</v>
+        <v>1419928.7399999967</v>
       </c>
       <c r="E8">
         <v>872.61</v>
       </c>
       <c r="F8">
-        <v>1431292.3500000006</v>
+        <v>1431116.01</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -7152,7 +7152,7 @@
         <v>0.6965939402580261</v>
       </c>
       <c r="O8">
-        <v>0.6964081099397869</v>
+        <v>0.6963873350360231</v>
       </c>
       <c r="P8">
         <v>0.6317542791366577</v>
@@ -7176,13 +7176,13 @@
         <v>2943.28</v>
       </c>
       <c r="D9">
-        <v>5109330.949999997</v>
+        <v>5110004.719999988</v>
       </c>
       <c r="E9">
         <v>2943.28</v>
       </c>
       <c r="F9">
-        <v>5109272.099999999</v>
+        <v>5107081.200000004</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -7216,13 +7216,13 @@
         <v>970.93</v>
       </c>
       <c r="D10">
-        <v>1190379.199999998</v>
+        <v>1160505.19</v>
       </c>
       <c r="E10">
         <v>970.93</v>
       </c>
       <c r="F10">
-        <v>1186057.9000000013</v>
+        <v>1161096.8499999999</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -7256,13 +7256,13 @@
         <v>272.61</v>
       </c>
       <c r="D11">
-        <v>472462.0000000018</v>
+        <v>472039.910000001</v>
       </c>
       <c r="E11">
         <v>272.61</v>
       </c>
       <c r="F11">
-        <v>472107.95000000065</v>
+        <v>472819.9899999998</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -7293,16 +7293,16 @@
         </is>
       </c>
       <c r="C12">
-        <v>114.65</v>
+        <v>115.89</v>
       </c>
       <c r="D12">
-        <v>202495.6600000001</v>
+        <v>195755.7500000005</v>
       </c>
       <c r="E12">
         <v>110.34</v>
       </c>
       <c r="F12">
-        <v>176056.72999999992</v>
+        <v>172393.4300000006</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -7327,7 +7327,7 @@
         <v>0.6553257405757904</v>
       </c>
       <c r="O12">
-        <v>0.6530525516122397</v>
+        <v>0.6541229435415905</v>
       </c>
       <c r="P12">
         <v>0.5647161602973938</v>
@@ -7348,16 +7348,16 @@
         </is>
       </c>
       <c r="C13">
-        <v>220.77</v>
+        <v>218.9</v>
       </c>
       <c r="D13">
-        <v>358195.0000000003</v>
+        <v>391518.54999999935</v>
       </c>
       <c r="E13">
         <v>214.57</v>
       </c>
       <c r="F13">
-        <v>368960.7099999988</v>
+        <v>370310.4100000006</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -7382,7 +7382,7 @@
         <v>0.8098851243654887</v>
       </c>
       <c r="O13">
-        <v>0.7402637658592744</v>
+        <v>0.7389471297125113</v>
       </c>
       <c r="P13">
         <v>0.5294176340103149</v>
@@ -7406,13 +7406,13 @@
         <v>2610.32</v>
       </c>
       <c r="D14">
-        <v>4398730.870000009</v>
+        <v>4401692.920000008</v>
       </c>
       <c r="E14">
         <v>2610.32</v>
       </c>
       <c r="F14">
-        <v>4400881.609999997</v>
+        <v>4401265.419999995</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -7446,13 +7446,13 @@
         <v>4092.56</v>
       </c>
       <c r="D15">
-        <v>4612887.960000006</v>
+        <v>4655078.979999998</v>
       </c>
       <c r="E15">
         <v>4092.56</v>
       </c>
       <c r="F15">
-        <v>4623988.199999998</v>
+        <v>4660354.21</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -7486,13 +7486,13 @@
         <v>275.65</v>
       </c>
       <c r="D16">
-        <v>454454.1599999994</v>
+        <v>453443.55000000016</v>
       </c>
       <c r="E16">
         <v>275.65</v>
       </c>
       <c r="F16">
-        <v>453997.5499999992</v>
+        <v>453614.39000000025</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -7526,13 +7526,13 @@
         <v>1505.95</v>
       </c>
       <c r="D17">
-        <v>2609095.2300000046</v>
+        <v>2608870.07</v>
       </c>
       <c r="E17">
         <v>1505.95</v>
       </c>
       <c r="F17">
-        <v>2608828.890000008</v>
+        <v>2609248.409999997</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -7563,16 +7563,16 @@
         </is>
       </c>
       <c r="C18">
-        <v>170.25</v>
+        <v>170.33</v>
       </c>
       <c r="D18">
-        <v>282227.7499999999</v>
+        <v>283652.3799999994</v>
       </c>
       <c r="E18">
         <v>167.51</v>
       </c>
       <c r="F18">
-        <v>279951.4500000005</v>
+        <v>280137.0900000003</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -7597,7 +7597,7 @@
         <v>0.9814960360527039</v>
       </c>
       <c r="O18">
-        <v>0.9815501190966867</v>
+        <v>0.9815527296914881</v>
       </c>
       <c r="P18">
         <v>0.9661091566085815</v>
@@ -7618,16 +7618,16 @@
         </is>
       </c>
       <c r="C19">
-        <v>807.71</v>
+        <v>806.14</v>
       </c>
       <c r="D19">
-        <v>1309712.8800000087</v>
+        <v>1335372.8400000012</v>
       </c>
       <c r="E19">
         <v>793.68</v>
       </c>
       <c r="F19">
-        <v>1221695.8700000027</v>
+        <v>1251665.8999999983</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -7652,7 +7652,7 @@
         <v>0.5739879906177521</v>
       </c>
       <c r="O19">
-        <v>0.573995562871005</v>
+        <v>0.5740174029920202</v>
       </c>
       <c r="P19">
         <v>0.5584376454353333</v>
@@ -7673,16 +7673,16 @@
         </is>
       </c>
       <c r="C20">
-        <v>470.62</v>
+        <v>469.33</v>
       </c>
       <c r="D20">
-        <v>734897.1999999968</v>
+        <v>781931.3800000009</v>
       </c>
       <c r="E20">
         <v>459.9</v>
       </c>
       <c r="F20">
-        <v>750244.2199999979</v>
+        <v>753835.8299999996</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -7707,7 +7707,7 @@
         <v>0.5485995511213938</v>
       </c>
       <c r="O20">
-        <v>0.573283185298977</v>
+        <v>0.5737625769305833</v>
       </c>
       <c r="P20">
         <v>0.49337705969810486</v>
@@ -7731,13 +7731,13 @@
         <v>738.25</v>
       </c>
       <c r="D21">
-        <v>877633.200000001</v>
+        <v>779971.2699999986</v>
       </c>
       <c r="E21">
         <v>738.25</v>
       </c>
       <c r="F21">
-        <v>901705.450000002</v>
+        <v>785411.4999999987</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -7768,16 +7768,16 @@
         </is>
       </c>
       <c r="C22">
-        <v>476.35</v>
+        <v>476.25</v>
       </c>
       <c r="D22">
-        <v>750668.7899999996</v>
+        <v>714505.2299999994</v>
       </c>
       <c r="E22">
         <v>476.33</v>
       </c>
       <c r="F22">
-        <v>752372.6999999979</v>
+        <v>703873.2100000003</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -7802,7 +7802,7 @@
         <v>0.4284673035144806</v>
       </c>
       <c r="O22">
-        <v>0.4284673035144806</v>
+        <v>0.42846730351448065</v>
       </c>
       <c r="P22">
         <v>0.4284673035144806</v>
@@ -7823,16 +7823,16 @@
         </is>
       </c>
       <c r="C23">
-        <v>475.21</v>
+        <v>475.37</v>
       </c>
       <c r="D23">
-        <v>801171.3399999978</v>
+        <v>816880.2600000006</v>
       </c>
       <c r="E23">
         <v>467.82</v>
       </c>
       <c r="F23">
-        <v>808915.1500000001</v>
+        <v>808832.0199999993</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         <v>0.6775287389755249</v>
       </c>
       <c r="O23">
-        <v>0.6276030359295445</v>
+        <v>0.6266021872298921</v>
       </c>
       <c r="P23">
         <v>0.46839380264282227</v>
@@ -7881,13 +7881,13 @@
         <v>759.24</v>
       </c>
       <c r="D24">
-        <v>1317595.4699999967</v>
+        <v>1317286.159999994</v>
       </c>
       <c r="E24">
         <v>759.24</v>
       </c>
       <c r="F24">
-        <v>1316914.5099999984</v>
+        <v>1317638.6099999982</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -7921,13 +7921,13 @@
         <v>2398.34</v>
       </c>
       <c r="D25">
-        <v>4161942.5100000016</v>
+        <v>4163072.9299999895</v>
       </c>
       <c r="E25">
         <v>2398.34</v>
       </c>
       <c r="F25">
-        <v>4162731.5000000102</v>
+        <v>4163707.969999989</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -7961,13 +7961,13 @@
         <v>2320.8</v>
       </c>
       <c r="D26">
-        <v>3507124.8299999936</v>
+        <v>3503571.78999999</v>
       </c>
       <c r="E26">
         <v>2320.8</v>
       </c>
       <c r="F26">
-        <v>3514969.899999995</v>
+        <v>3504827.670000001</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -8001,13 +8001,13 @@
         <v>1297.8</v>
       </c>
       <c r="D27">
-        <v>2204445.7400000067</v>
+        <v>2204369.89</v>
       </c>
       <c r="E27">
         <v>1297.8</v>
       </c>
       <c r="F27">
-        <v>2204028.2899999986</v>
+        <v>2203776.8700000006</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -8041,13 +8041,13 @@
         <v>238.47</v>
       </c>
       <c r="D28">
-        <v>402066.18999999965</v>
+        <v>402128.86999999906</v>
       </c>
       <c r="E28">
         <v>238.47</v>
       </c>
       <c r="F28">
-        <v>402468.99000000005</v>
+        <v>402039.59999999905</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -8081,13 +8081,13 @@
         <v>799.84</v>
       </c>
       <c r="D29">
-        <v>1379738.2499999984</v>
+        <v>1378617.7299999993</v>
       </c>
       <c r="E29">
         <v>799.84</v>
       </c>
       <c r="F29">
-        <v>1378389.9100000053</v>
+        <v>1378742.9999999932</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -8121,13 +8121,13 @@
         <v>575.41</v>
       </c>
       <c r="D30">
-        <v>973503.4599999986</v>
+        <v>972390.6400000018</v>
       </c>
       <c r="E30">
         <v>575.41</v>
       </c>
       <c r="F30">
-        <v>973429.3599999979</v>
+        <v>973099.9899999995</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -8161,13 +8161,13 @@
         <v>301.74</v>
       </c>
       <c r="D31">
-        <v>489840.9200000032</v>
+        <v>488296.4300000003</v>
       </c>
       <c r="E31">
         <v>301.74</v>
       </c>
       <c r="F31">
-        <v>487262.08000000083</v>
+        <v>488103.34000000014</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -8201,13 +8201,13 @@
         <v>451.42</v>
       </c>
       <c r="D32">
-        <v>764302.9500000017</v>
+        <v>763551.4800000003</v>
       </c>
       <c r="E32">
         <v>451.42</v>
       </c>
       <c r="F32">
-        <v>764168.6800000012</v>
+        <v>763171.9400000019</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -8241,13 +8241,13 @@
         <v>1432.54</v>
       </c>
       <c r="D33">
-        <v>2381664.61</v>
+        <v>2379893.2999999984</v>
       </c>
       <c r="E33">
         <v>1432.54</v>
       </c>
       <c r="F33">
-        <v>2383809.0100000016</v>
+        <v>2379380.0700000026</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>

</xml_diff>